<commit_message>
Publish reviewed Tang Tianqi profile with validated site and workbook exports
</commit_message>
<xml_diff>
--- a/site/exports/hit-energy.xlsx
+++ b/site/exports/hit-energy.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$203</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$209</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -453,8 +453,8 @@
     <col width="32.2" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="37.8" customWidth="1" min="7" max="7"/>
-    <col width="40.59999999999999" customWidth="1" min="8" max="8"/>
-    <col width="23.8" customWidth="1" min="9" max="9"/>
+    <col width="47.59999999999999" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
@@ -2106,8 +2106,61 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>无具体论文或专著书目；不由搜索摘要增补。；本硕博就读，不等于明确获授学位；学位及授位日期均未知。；2024来源职称不认证2026当前职位。；来源记载职业信息：2020；申请学校预留师资博士后。申请事件不是博士后入职。 来源：https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm；来源记载职业信息：2020-10-28；第三届优秀博士研究生预留师资博士后入选名单。学科原文：动力工程及工程热物理。按同名、学科与简介2020申请相互参照，非独立唯一身份认证；选拔公示不证明实际在站或学位，不转换为正式在站日期或本科/硕士专业。 来源：https://hitgs.hit.edu.cn/2020/1028/c17343a329755/page.htm；来源记载职业信息：时间未述；协助指导本科生参加全国大学生节能减排社会实践与科技竞赛、“零碳未来创新大赛”等项目，获特等奖2项。合并表述2项，不拆分赛事各自奖项数，不作个人论文作品。 来源：https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm；教师简介报道发布于2024-03-26，文末署期2024-03-24；选拔公示发布于2020-10-28。这些历史来源不证明2026当前任职或博士后在站。；旧名录2026-10-23收录于能源与环境工程研究所，未提供个人主页且未标独立个人主页身份认证；本轮不修改原名录、不声称新读。校区仅沿用同日既有单位证据。；教育院校985、地域与洲本批不推补；荷兰仅保留来源国家原文。</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>尚无已核实个人主页；以下为学校官方活动报道与选拔公示，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>官方活动报道（含教师简介）：https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm；官方预留师资博士后选拔公示：https://hitgs.hit.edu.cn/2020/1028/c17343a329755/page.htm</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K31"/>
+  <autoFilter ref="A1:K32"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -2150,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S203"/>
+  <dimension ref="A1:S209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -14815,8 +14868,340 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr"/>
+      <c r="F204" s="2" t="inlineStr"/>
+      <c r="G204" s="2" t="inlineStr"/>
+      <c r="H204" s="2" t="inlineStr"/>
+      <c r="I204" s="2" t="inlineStr"/>
+      <c r="J204" s="2" t="inlineStr"/>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L204" s="2" t="inlineStr"/>
+      <c r="M204" s="2" t="inlineStr"/>
+      <c r="N204" s="2" t="inlineStr"/>
+      <c r="O204" s="2" t="inlineStr">
+        <is>
+          <t>来源原文为本硕博均就读哈尔滨工业大学；本条仅本科学习阶段，不认定获授学位。专业、阶段起止与授位日期均未知。</t>
+        </is>
+      </c>
+      <c r="P204" s="2" t="inlineStr"/>
+      <c r="Q204" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R204" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S204" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr"/>
+      <c r="F205" s="2" t="inlineStr"/>
+      <c r="G205" s="2" t="inlineStr"/>
+      <c r="H205" s="2" t="inlineStr"/>
+      <c r="I205" s="2" t="inlineStr"/>
+      <c r="J205" s="2" t="inlineStr"/>
+      <c r="K205" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L205" s="2" t="inlineStr"/>
+      <c r="M205" s="2" t="inlineStr"/>
+      <c r="N205" s="2" t="inlineStr"/>
+      <c r="O205" s="2" t="inlineStr">
+        <is>
+          <t>来源原文为本硕博均就读哈尔滨工业大学；本条仅硕士学习阶段，不认定获授学位。专业、阶段起止与授位日期均未知。</t>
+        </is>
+      </c>
+      <c r="P205" s="2" t="inlineStr"/>
+      <c r="Q205" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R205" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S205" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr"/>
+      <c r="F206" s="2" t="inlineStr"/>
+      <c r="G206" s="2" t="inlineStr"/>
+      <c r="H206" s="2" t="inlineStr"/>
+      <c r="I206" s="2" t="inlineStr"/>
+      <c r="J206" s="2" t="inlineStr"/>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L206" s="2" t="inlineStr"/>
+      <c r="M206" s="2" t="inlineStr"/>
+      <c r="N206" s="2" t="inlineStr"/>
+      <c r="O206" s="2" t="inlineStr">
+        <is>
+          <t>来源原文为本硕博均就读哈尔滨工业大学；本条仅博士学习阶段，不认定获授学位。专业、阶段起止与授位日期均未知。</t>
+        </is>
+      </c>
+      <c r="P206" s="2" t="inlineStr"/>
+      <c r="Q206" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R206" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S206" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>joint_training</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr"/>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>埃因霍温理工大学</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr"/>
+      <c r="F207" s="2" t="inlineStr"/>
+      <c r="G207" s="2" t="inlineStr"/>
+      <c r="H207" s="2" t="inlineStr"/>
+      <c r="I207" s="2" t="inlineStr"/>
+      <c r="J207" s="2" t="inlineStr"/>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L207" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M207" s="2" t="inlineStr"/>
+      <c r="N207" s="2" t="inlineStr"/>
+      <c r="O207" s="2" t="inlineStr">
+        <is>
+          <t>来源记载2019年赴荷兰埃因霍温理工大学联培；机构原文：荷兰埃因霍温理工大学；国家原文：荷兰。2019仅事件年份，不是起止日期；阶段未知，不推博士联培或独立学位，不据校名补地域分类。</t>
+        </is>
+      </c>
+      <c r="P207" s="2" t="inlineStr"/>
+      <c r="Q207" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R207" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S207" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>讲师</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr"/>
+      <c r="F208" s="2" t="inlineStr"/>
+      <c r="G208" s="2" t="inlineStr"/>
+      <c r="H208" s="2" t="inlineStr"/>
+      <c r="I208" s="2" t="inlineStr"/>
+      <c r="J208" s="2" t="inlineStr"/>
+      <c r="K208" s="2" t="inlineStr"/>
+      <c r="L208" s="2" t="inlineStr"/>
+      <c r="M208" s="2" t="inlineStr"/>
+      <c r="N208" s="2" t="inlineStr"/>
+      <c r="O208" s="2" t="inlineStr">
+        <is>
+          <t>2024-03-26报道记载能源科学与工程学院讲师；仅为该来源时点职称，不认证2026当前职位；任职起止未知。</t>
+        </is>
+      </c>
+      <c r="P208" s="2" t="inlineStr"/>
+      <c r="Q208" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R208" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S208" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>毕业留校工作</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr"/>
+      <c r="F209" s="2" t="inlineStr"/>
+      <c r="G209" s="2" t="inlineStr"/>
+      <c r="H209" s="2" t="inlineStr"/>
+      <c r="I209" s="2" t="inlineStr"/>
+      <c r="J209" s="2" t="inlineStr"/>
+      <c r="K209" s="2" t="inlineStr"/>
+      <c r="L209" s="2" t="inlineStr"/>
+      <c r="M209" s="2" t="inlineStr"/>
+      <c r="N209" s="2" t="inlineStr"/>
+      <c r="O209" s="2" t="inlineStr">
+        <is>
+          <t>来源事件月份：2021-07，毕业留校工作；仅event_date，不是聘任任期、讲师或博士后聘任起点，不是授位日期；毕业学位阶段原句未单列，start/end均未知。</t>
+        </is>
+      </c>
+      <c r="P209" s="2" t="inlineStr"/>
+      <c r="Q209" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R209" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S209" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S203"/>
+  <autoFilter ref="A1:S209"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -15021,6 +15406,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q201" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q202" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q203" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q204" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q205" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q206" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q207" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q208" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q209" r:id="rId209"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15032,7 +15423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -15705,8 +16096,58 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>来源导师（阶段未知）</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>来源称导师何玉荣教授；本硕博就读概述后的导师括注，未明确仅博士或覆盖全部阶段；只保一条阶段未知的来源导师关系。 关系起止未知，未核学位论文原件；不绑定任一教育事件，不认定全阶段或博士导师，人物身份与现职未独立匹配，无身份导航。</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>来源头衔为教授；当前任职未独立核验，无身份或主页导航。</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L12"/>
+  <autoFilter ref="A1:L13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
@@ -15719,6 +16160,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17764,7 +18206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -21476,8 +21918,156 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>hit-tangtianqi-biography-20261030</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>学校官方报道/公示正文有界复读，非个人主页与当前人事认证。；independent_normal_web_official_article_body_read</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>hit-tangtianqi-notice-20261030</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>https://hitgs.hit.edu.cn/2020/1028/c17343a329755/page.htm</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>学校官方报道/公示正文有界复读，非个人主页与当前人事认证。；independent_normal_web_official_article_body_read</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>hit-tangtianqi-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有名录身份与能源与环境工程研究所目录归组；无个人主页，不声称本轮重读。</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>唐天琪</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>hit-tangtianqi-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位校区证据复用harbin；非本轮重新读取。</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G100"/>
+  <autoFilter ref="A1:G104"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -21578,6 +22168,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish six reviewed HIT faculty profiles and validated exports
</commit_message>
<xml_diff>
--- a/site/exports/hit-energy.xlsx
+++ b/site/exports/hit-energy.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$209</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,7 @@
     <col width="32.2" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="37.8" customWidth="1" min="7" max="7"/>
-    <col width="47.59999999999999" customWidth="1" min="8" max="8"/>
+    <col width="54.59999999999999" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
@@ -2159,8 +2159,326 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>学习起止、授位日期、专业和硕士经历均未明；本人导师未知。；来源职务仅报道时点，非2026现职认证或聘期。；没有已核具体论文或专著，不把统计论文数当书目。；2017通知页头2017-11-24、拟会议2017-11-25、落款2017-12-23，存在日期冲突；保留不修正、不调序，不推聘期。；来源记载职业信息：内容：国家自然科学优秀青年科学基金；日期：2017。来源：https://www.nwpu.edu.cn/info/1039/2890.htm；来源记载职业信息：内容：教育部科学技术进步一等奖；日期：2015。来源：https://www.nwpu.edu.cn/info/1039/2890.htm；来源记载职业信息：内容：黑龙江省自然科学二等奖；日期：2014。来源：https://www.nwpu.edu.cn/info/1039/2890.htm；来源记载职业信息：内容：冲压发动机领域“兴洲奖”获得者。来源：https://www.nwpu.edu.cn/info/1039/2890.htm；来源记载职业信息：内容：航天第三专业信息网发动机控制专业委员会委员；《空气动力学报》和《实验流体力学》青年编委；3个国际期刊编委；来源记载时点：2017-11-24。来源：https://www.nwpu.edu.cn/info/1039/2890.htm；来源记载职业信息：内容：国家杰青；中国工程热物理学会吴仲华优秀青年学者奖、第三届“兴洲奖”、教育部技术进步一等奖、国防技术发明二等奖、爱思唯尔高被引学者等荣誉；来源记载时点：2022-05-16；限制说明：2017与2022两来源奖名表述保留，不计为不重复奖项总数。。来源：https://www.ncepu.edu.cn/xshd/f1015865691c45f6ac9b48dd423957e6.htm；来源记载职业信息：内容：第八届空气动力学学会理事；中国空天动力联合会发动机控制组专业委员会主任；《气动研究与试验》副主编；《推进技术》《航空学报》中/英文版、《实验流体力学》《空气动力学学报》《气体物理》等6个期刊编委/青年编委；来源记载时点：2022-05-16。来源：https://www.ncepu.edu.cn/xshd/f1015865691c45f6ac9b48dd423957e6.htm；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。；2022-05-16为讲座通知刊发日期，拟讲座时间2022-05-17；计划通知不确认活动已举办。</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>官方职业报道或报告人简介：https://news.hit.edu.cn/2025/0522/c1510a238003/page.htm；官方职业报道或报告人简介：https://www.nwpu.edu.cn/info/1039/2890.htm；官方职业报道或报告人简介：https://www.ncepu.edu.cn/xshd/f1015865691c45f6ac9b48dd423957e6.htm</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>本科、硕士及博士授位时间未知。；职业新闻所载团队关系不推个人博士导师。；同名论文结合清华读博及等离子体方向关联，不宣称独立唯一身份认证或论文全文核验。；德国任职单位、具体起止未知；来源职务不认证2026此刻在职。；来源记载职业信息：内容：入选洪堡学者。来源：https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm；来源记载职业信息：内容：国家级青年人才；来源记载时点：2026-03-18。来源：https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm；来源记载职业信息：内容：2017年度博士生指导教师遴选通过，申报学科动力工程及工程热物理；通知说明新增校内导师从2018年起招收指导博士研究生；日期：2017-04-26；限制说明：是本人指导资格，非本人学位/导师。。来源：https://hitgs.hit.edu.cn/2017/0426/c17413a317511/page.htm；来源记载职业信息：内容：通知拟安排2018年7月9日至13日《等离子体物理与工程应用》课程，由朱悉铭与宁中喜共同主持；来源记载时点：2018-07-02；限制说明：通知安排，不据此确认活动已举办；2018-07-02仅为通知发布日期。。来源：https://hitgs.hit.edu.cn/2018/0702/c17506a330002/page.htm；来源记载职业信息：内容：传记回顾其参加首届青年学者神舟论坛时已发表SCI论文40余篇。；来源记载时点：2026-03-18；限制说明：彼时统计，不是2026当前总量，不生成具名作品。。来源：https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>官方职业报道或报告人简介：https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm；官方公开论文目录：https://newetds.lib.tsinghua.edu.cn/qh/paper/summary?dbCode=ETDQH&amp;sysId=189075；官方指导资格通知：https://hitgs.hit.edu.cn/2017/0426/c17413a317511/page.htm；官方课程计划通知：https://hitgs.hit.edu.cn/2018/0702/c17506a330002/page.htm</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>阶段标签不推授位，学历日期/专业/本人导师未知。；两个访问研究经历起止和职衔未知，非授位。；职务是2024来源记载，不认证2026当前在职；深圳市重点实验室名称未明。；原简介专业委员会句与期刊清单相连疑缺词，不修复为未经证实任职。；教材/论文仅统计无书目，不生成具体作品。；来源记载职业信息：内容：获教育部自然科学二等奖1项，黑龙江省自然科学二等奖2项。。来源：https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm；来源记载职业信息：内容：国家自然科学基金委通讯评议专家；国家高新技术企业专家咨询指导委员会委员；教育部学位论文通讯评议专家；广东省先进核能人工智能与虚拟现实工程技术研究中心工程技术委员会委员；；来源记载时点：2024-05-29。来源：https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm；来源记载职业信息：内容：AIChE Journal, Physics of Fluids, Energy and Fuel, Fuel, Powder Technology, Advanced Powder Technology, Chemical Engineering Research and Design, Chemical Engineering and Technology, Canadian Journal of Chemical Engineering, Petroleum Science, Flow Turbulence and Combustion, Annals of Nuclear Energy，《工程热物理学报》，《西北工业大学学报》，《东南大学学报》等三十余个国际及国内期刊审稿人。；来源记载时点：2024-05-29；限制说明：前接“第十届中国核物理学会反应堆物理与核材料专业委员会”但未给完整职责，原片段保留，不自补委员身份或改变期刊原名。。来源：https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm；来源记载职业信息：内容：2024年简介称近年来出版教材2部、发表SCI检索论文九十余篇；负责某部委科技重点基金、国家自然科学基金面上等科研项目共十余项。；来源记载时点：2024-05-29；限制说明：原时点总量，不编造具体书目/项目，不将十余项分配给每一类别。。来源：https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>官方职业报道或报告人简介：https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>王子傲</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>授位院校、专业、日期未知；本人导师未知；教育分段未知；现职起止未知；无具名论文书目；研究生导师为其指导资格，不转换本人导师关系；SCI40篇为源截至日期自述总量，不造40条作品；两页同名HIT职业与学院/既有名录闭合，未借用同名招生学生记录；来源记载职业信息：姓名：王子傲；机构：哈尔滨工业大学；来源角色：助理教授、研究生导师、兼职辅导员；资格：工学博士；研究方向：超声速流动机理、监测及控制方法；项目概述：角色：主持；数量：7；计数单位：项项目；举例类别：国家自然科学基金、中国博士后基金面上项目、航空科学基金；范围限制：等7项总量，非每类7项；截至来源简介；成果统计：检索口径：SCI；数量：40；计数单位：篇；统计时点：累计；截至来源简介；领域：流体力学、航空航天；荣誉：第九届中国科协青年人才托举工程、2023年度全球前2%科学家榜单；学术服务：机构或期刊：processes；角色：客座主编、机构或期刊：中国航天第三专业信息网专委会；角色：青年委员、机构或期刊：海军航空大学学报；角色：期刊青年编委；计划活动（非已举办确认）：标题：一研为定——如何为研究生学习做好准备；计划时间：2024-03-31T15:30；来源状态：活动通知计划，不声称已举办。各汇总为来源时点合述，不生成逐项论文或推定任职起止；计划活动不确认已举办。来源：https://future.hit.edu.cn/2024/0330/c16314a341158/page.htm；来源记载教学资格：姓名：王子傲；单位：能源科学与工程学院；资格认证：本科主讲教师授课资格认证；课程：飞行器动力系统及环境工程；通过日期：2024-11-05。通过日2024-11-05与公布日2024-11-06不同；不构成学历。来源：https://hituc.hit.edu.cn/2024/1106/c17860a358734/page.htm；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>官方职业报道或报告人简介：https://future.hit.edu.cn/2024/0330/c16314a341158/page.htm；官方教学资格通知：https://hituc.hit.edu.cn/2024/1106/c17860a358734/page.htm</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>各学位专业未知；本人导师未知；工作角色开始结束日期未知；无具名作品信息；网址2023/0919不替代可见发布日期2022-11-08。；双学士作为来源合并事件保留数量2；未提供两专业，不拆造不同专业学位。；来源记载职业信息：来源角色：能源科学与工程学院副院长、教授、博导；来源学位概述：年份：2006；机构：哈尔滨工业大学；称谓：双学士、年份：2008；机构：哈尔滨工业大学；称谓：硕士、年份：2012；机构：普瓦提埃大学；国家原文：法国；称谓：博士；原文工作顺序：CNRS-普瓦提埃大学、西班牙塞维利亚大学、CNRS-洛林大学；回国入职年份：2017；回国入职原文：回国入职哈工大；职业荣誉：年份：2021；称谓：哈工大青年科学家工作室带头人；动作：获批；计划活动（非已举办确认）：日期：2022-11-12；时间：18:30；主题：欧洲地区留学经验分享会（二）；本人报告主题：法国留学经历。各汇总为来源时点合述，不生成逐项论文或推定任职起止；计划活动不确认已举办。来源：https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。；来源可见发布日期与落款为2022-11-08，网址路径含2023/0919；保留差异，不把路径年份当发布日期。旧威海同名名录不合并。</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>官方职业报道或报告人简介：https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>各学位专业未知；本人导师未知；工作角色开始结束日期未知；无具名作品信息；未给专业/本人导师/聘任起止；不由博导推其导师身份。；来源记载职业信息：来源角色：能源学院教授、博导；人才项目：国家级青年人才计划项目；动作：入选；来源学位概述：年份：2012；机构：西安交通大学；称谓：学士、年份：2015；机构：西安交通大学；称谓：硕士、年份：2019；机构：香港大学；称谓：博士；计划活动（非已举办确认）：日期：2024-11-03；时间：18:30；主题：香港地区留学经验分享会；本人报告主题：香港留学经历。各汇总为来源时点合述，不生成逐项论文或推定任职起止；计划活动不确认已举办。来源：https://future.hit.edu.cn/2024/1029/c16314a357783/page.htm；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>官方职业报道或报告人简介：https://future.hit.edu.cn/2024/1029/c16314a357783/page.htm</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K32"/>
+  <autoFilter ref="A1:K38"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -2203,7 +2521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S209"/>
+  <dimension ref="A1:S240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -15200,8 +15518,1731 @@
         </is>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr"/>
+      <c r="F210" s="2" t="inlineStr"/>
+      <c r="G210" s="2" t="inlineStr"/>
+      <c r="H210" s="2" t="inlineStr"/>
+      <c r="I210" s="2" t="inlineStr"/>
+      <c r="J210" s="2" t="inlineStr"/>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L210" s="2" t="inlineStr"/>
+      <c r="M210" s="2" t="inlineStr"/>
+      <c r="N210" s="2" t="inlineStr"/>
+      <c r="O210" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；学习阶段：本科。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P210" s="2" t="inlineStr"/>
+      <c r="Q210" s="3" t="inlineStr">
+        <is>
+          <t>https://news.hit.edu.cn/2025/0522/c1510a238003/page.htm</t>
+        </is>
+      </c>
+      <c r="R210" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S210" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr"/>
+      <c r="F211" s="2" t="inlineStr"/>
+      <c r="G211" s="2" t="inlineStr"/>
+      <c r="H211" s="2" t="inlineStr"/>
+      <c r="I211" s="2" t="inlineStr"/>
+      <c r="J211" s="2" t="inlineStr"/>
+      <c r="K211" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L211" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M211" s="2" t="inlineStr"/>
+      <c r="N211" s="2" t="inlineStr"/>
+      <c r="O211" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；学习阶段：博士；来源层次：博士；限制说明：2025原句为包括常军涛在内的三位教师合述在哈工大从本科生成长为博士，非单独教育履历或原文获授措辞；2017报告人简介另明确常军涛本人博士资格。两处共同支撑来源记载资格，非证书查验，不推授位年份、专业或硕士经历。。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P211" s="2" t="inlineStr"/>
+      <c r="Q211" s="3" t="inlineStr">
+        <is>
+          <t>https://news.hit.edu.cn/2025/0522/c1510a238003/page.htm</t>
+        </is>
+      </c>
+      <c r="R211" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S211" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr"/>
+      <c r="F212" s="2" t="inlineStr"/>
+      <c r="G212" s="2" t="inlineStr"/>
+      <c r="H212" s="2" t="inlineStr"/>
+      <c r="I212" s="2" t="inlineStr"/>
+      <c r="J212" s="2" t="inlineStr"/>
+      <c r="K212" s="2" t="inlineStr"/>
+      <c r="L212" s="2" t="inlineStr"/>
+      <c r="M212" s="2" t="inlineStr"/>
+      <c r="N212" s="2" t="inlineStr"/>
+      <c r="O212" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位原文：能源科学与工程学院；来源角色：教授；来源记载时点：2025-05-21。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。 报道刊发于2025-05-22，会议发生于2025-05-21；二者不作为任职起点。</t>
+        </is>
+      </c>
+      <c r="P212" s="2" t="inlineStr"/>
+      <c r="Q212" s="3" t="inlineStr">
+        <is>
+          <t>https://news.hit.edu.cn/2025/0522/c1510a238003/page.htm</t>
+        </is>
+      </c>
+      <c r="R212" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S212" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>教授、博士生导师</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr"/>
+      <c r="F213" s="2" t="inlineStr"/>
+      <c r="G213" s="2" t="inlineStr"/>
+      <c r="H213" s="2" t="inlineStr"/>
+      <c r="I213" s="2" t="inlineStr"/>
+      <c r="J213" s="2" t="inlineStr"/>
+      <c r="K213" s="2" t="inlineStr"/>
+      <c r="L213" s="2" t="inlineStr"/>
+      <c r="M213" s="2" t="inlineStr"/>
+      <c r="N213" s="2" t="inlineStr"/>
+      <c r="O213" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；来源角色：教授、博士生导师；来源记载时点：2017-11-24；限制说明：2017通知页头2017-11-24、拟会议2017-11-25、落款2017-12-23，存在日期冲突；保留不修正、不调序，不推聘期。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P213" s="2" t="inlineStr"/>
+      <c r="Q213" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nwpu.edu.cn/info/1039/2890.htm</t>
+        </is>
+      </c>
+      <c r="R213" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S213" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>清华大学</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr"/>
+      <c r="F214" s="2" t="inlineStr"/>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>核科学与技术</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr"/>
+      <c r="I214" s="2" t="inlineStr"/>
+      <c r="J214" s="2" t="inlineStr"/>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L214" s="2" t="inlineStr"/>
+      <c r="M214" s="2" t="inlineStr"/>
+      <c r="N214" s="2" t="inlineStr"/>
+      <c r="O214" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：清华大学；学习阶段：博士；来源层次：博士；专业：核科学与技术；院系原文：032 工物系；答辩日期：2009-12-24；限制说明：HIT职业传记明确清华读博，清华公开论文元数据同名同研究领域相互参照；目录学位=博士标识论文层次，暂不升级授位确认；答辩日单独保留。。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。 同名、清华读博及等离子体方向有界对应，非独立唯一身份认证。</t>
+        </is>
+      </c>
+      <c r="P214" s="2" t="inlineStr"/>
+      <c r="Q214" s="3" t="inlineStr">
+        <is>
+          <t>https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm</t>
+        </is>
+      </c>
+      <c r="R214" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S214" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>加入团队</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr"/>
+      <c r="F215" s="2" t="inlineStr"/>
+      <c r="G215" s="2" t="inlineStr"/>
+      <c r="H215" s="2" t="inlineStr"/>
+      <c r="I215" s="2" t="inlineStr"/>
+      <c r="J215" s="2" t="inlineStr"/>
+      <c r="K215" s="2" t="inlineStr"/>
+      <c r="L215" s="2" t="inlineStr"/>
+      <c r="M215" s="2" t="inlineStr"/>
+      <c r="N215" s="2" t="inlineStr"/>
+      <c r="O215" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位原文：能源科学与工程学院于达仁教授团队；来源角色：加入团队；事件年份：2017；限制说明：加入团队事件，不推教授聘任时间；于达仁为团队负责人，不建立博士导师关系。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P215" s="2" t="inlineStr"/>
+      <c r="Q215" s="3" t="inlineStr">
+        <is>
+          <t>https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm</t>
+        </is>
+      </c>
+      <c r="R215" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S215" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>等离子体技术工作</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr"/>
+      <c r="E216" s="2" t="inlineStr"/>
+      <c r="F216" s="2" t="inlineStr"/>
+      <c r="G216" s="2" t="inlineStr"/>
+      <c r="H216" s="2" t="inlineStr"/>
+      <c r="I216" s="2" t="inlineStr"/>
+      <c r="J216" s="2" t="inlineStr"/>
+      <c r="K216" s="2" t="inlineStr"/>
+      <c r="L216" s="2" t="inlineStr"/>
+      <c r="M216" s="2" t="inlineStr"/>
+      <c r="N216" s="2" t="inlineStr"/>
+      <c r="O216" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：国家原文：德国；来源角色：等离子体技术工作；原文时长：3年；限制说明：原文以参加首届论坛时回顾3年，不推起止或单位。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P216" s="2" t="inlineStr"/>
+      <c r="Q216" s="3" t="inlineStr">
+        <is>
+          <t>https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm</t>
+        </is>
+      </c>
+      <c r="R216" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S216" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr"/>
+      <c r="F217" s="2" t="inlineStr"/>
+      <c r="G217" s="2" t="inlineStr"/>
+      <c r="H217" s="2" t="inlineStr"/>
+      <c r="I217" s="2" t="inlineStr"/>
+      <c r="J217" s="2" t="inlineStr"/>
+      <c r="K217" s="2" t="inlineStr"/>
+      <c r="L217" s="2" t="inlineStr"/>
+      <c r="M217" s="2" t="inlineStr"/>
+      <c r="N217" s="2" t="inlineStr"/>
+      <c r="O217" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；来源角色：教授；来源记载时点：2017-04-26。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P217" s="2" t="inlineStr"/>
+      <c r="Q217" s="3" t="inlineStr">
+        <is>
+          <t>https://hitgs.hit.edu.cn/2017/0426/c17413a317511/page.htm</t>
+        </is>
+      </c>
+      <c r="R217" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S217" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr"/>
+      <c r="F218" s="2" t="inlineStr"/>
+      <c r="G218" s="2" t="inlineStr"/>
+      <c r="H218" s="2" t="inlineStr"/>
+      <c r="I218" s="2" t="inlineStr"/>
+      <c r="J218" s="2" t="inlineStr"/>
+      <c r="K218" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L218" s="2" t="inlineStr"/>
+      <c r="M218" s="2" t="inlineStr"/>
+      <c r="N218" s="2" t="inlineStr"/>
+      <c r="O218" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；院系原文：能源科学与工程学院；学习阶段：本科；来源层次：本科；限制说明：来源仅列本科/硕士/博士阶段，没有明确获得学位措辞；不由博导推本人博士授位。。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P218" s="2" t="inlineStr"/>
+      <c r="Q218" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R218" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S218" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr"/>
+      <c r="F219" s="2" t="inlineStr"/>
+      <c r="G219" s="2" t="inlineStr"/>
+      <c r="H219" s="2" t="inlineStr"/>
+      <c r="I219" s="2" t="inlineStr"/>
+      <c r="J219" s="2" t="inlineStr"/>
+      <c r="K219" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L219" s="2" t="inlineStr"/>
+      <c r="M219" s="2" t="inlineStr"/>
+      <c r="N219" s="2" t="inlineStr"/>
+      <c r="O219" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；院系原文：能源科学与工程学院；学习阶段：硕士；来源层次：硕士；限制说明：来源仅列本科/硕士/博士阶段，没有明确获得学位措辞；不由博导推本人博士授位。。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P219" s="2" t="inlineStr"/>
+      <c r="Q219" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R219" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S219" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr"/>
+      <c r="F220" s="2" t="inlineStr"/>
+      <c r="G220" s="2" t="inlineStr"/>
+      <c r="H220" s="2" t="inlineStr"/>
+      <c r="I220" s="2" t="inlineStr"/>
+      <c r="J220" s="2" t="inlineStr"/>
+      <c r="K220" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L220" s="2" t="inlineStr"/>
+      <c r="M220" s="2" t="inlineStr"/>
+      <c r="N220" s="2" t="inlineStr"/>
+      <c r="O220" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；院系原文：能源科学与工程学院；学习阶段：博士；来源层次：博士；限制说明：来源仅列本科/硕士/博士阶段，没有明确获得学位措辞；不由博导推本人博士授位。。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P220" s="2" t="inlineStr"/>
+      <c r="Q220" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R220" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S220" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>visiting_research</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr"/>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>科罗拉多矿业大学</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr"/>
+      <c r="F221" s="2" t="inlineStr"/>
+      <c r="G221" s="2" t="inlineStr"/>
+      <c r="H221" s="2" t="inlineStr"/>
+      <c r="I221" s="2" t="inlineStr"/>
+      <c r="J221" s="2" t="inlineStr"/>
+      <c r="K221" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L221" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M221" s="2" t="inlineStr"/>
+      <c r="N221" s="2" t="inlineStr"/>
+      <c r="O221" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：科罗拉多矿业大学；限制说明：来源明确访问研究，不是学位；未给日期或具体职位。。非独立授位经历。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P221" s="2" t="inlineStr"/>
+      <c r="Q221" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R221" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S221" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>visiting_research</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr"/>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>普林斯顿大学</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr"/>
+      <c r="F222" s="2" t="inlineStr"/>
+      <c r="G222" s="2" t="inlineStr"/>
+      <c r="H222" s="2" t="inlineStr"/>
+      <c r="I222" s="2" t="inlineStr"/>
+      <c r="J222" s="2" t="inlineStr"/>
+      <c r="K222" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L222" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M222" s="2" t="inlineStr"/>
+      <c r="N222" s="2" t="inlineStr"/>
+      <c r="O222" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：普林斯顿大学；限制说明：来源明确访问研究，不是学位；未给日期或具体职位。。非独立授位经历。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P222" s="2" t="inlineStr"/>
+      <c r="Q222" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R222" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S222" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>教授、博士生导师</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr"/>
+      <c r="F223" s="2" t="inlineStr"/>
+      <c r="G223" s="2" t="inlineStr"/>
+      <c r="H223" s="2" t="inlineStr"/>
+      <c r="I223" s="2" t="inlineStr"/>
+      <c r="J223" s="2" t="inlineStr"/>
+      <c r="K223" s="2" t="inlineStr"/>
+      <c r="L223" s="2" t="inlineStr"/>
+      <c r="M223" s="2" t="inlineStr"/>
+      <c r="N223" s="2" t="inlineStr"/>
+      <c r="O223" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位原文：能源科学与工程学院；来源角色：教授、博士生导师；来源记载时点：2024-05-29。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P223" s="2" t="inlineStr"/>
+      <c r="Q223" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R223" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S223" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>院长</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr"/>
+      <c r="E224" s="2" t="inlineStr"/>
+      <c r="F224" s="2" t="inlineStr"/>
+      <c r="G224" s="2" t="inlineStr"/>
+      <c r="H224" s="2" t="inlineStr"/>
+      <c r="I224" s="2" t="inlineStr"/>
+      <c r="J224" s="2" t="inlineStr"/>
+      <c r="K224" s="2" t="inlineStr"/>
+      <c r="L224" s="2" t="inlineStr"/>
+      <c r="M224" s="2" t="inlineStr"/>
+      <c r="N224" s="2" t="inlineStr"/>
+      <c r="O224" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：单位原文：先进核能与新能源研究院（中广核-哈工大）；来源角色：院长；来源记载时点：2024-05-29。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P224" s="2" t="inlineStr"/>
+      <c r="Q224" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R224" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S224" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>副主任</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr"/>
+      <c r="E225" s="2" t="inlineStr"/>
+      <c r="F225" s="2" t="inlineStr"/>
+      <c r="G225" s="2" t="inlineStr"/>
+      <c r="H225" s="2" t="inlineStr"/>
+      <c r="I225" s="2" t="inlineStr"/>
+      <c r="J225" s="2" t="inlineStr"/>
+      <c r="K225" s="2" t="inlineStr"/>
+      <c r="L225" s="2" t="inlineStr"/>
+      <c r="M225" s="2" t="inlineStr"/>
+      <c r="N225" s="2" t="inlineStr"/>
+      <c r="O225" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：单位原文：黑龙江省新型储能材料与储能过程研究重点实验室；来源角色：副主任；来源记载时点：2024-05-29。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P225" s="2" t="inlineStr"/>
+      <c r="Q225" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R225" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S225" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>副主任</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr"/>
+      <c r="E226" s="2" t="inlineStr"/>
+      <c r="F226" s="2" t="inlineStr"/>
+      <c r="G226" s="2" t="inlineStr"/>
+      <c r="H226" s="2" t="inlineStr"/>
+      <c r="I226" s="2" t="inlineStr"/>
+      <c r="J226" s="2" t="inlineStr"/>
+      <c r="K226" s="2" t="inlineStr"/>
+      <c r="L226" s="2" t="inlineStr"/>
+      <c r="M226" s="2" t="inlineStr"/>
+      <c r="N226" s="2" t="inlineStr"/>
+      <c r="O226" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：单位原文：深圳市重点实验室；来源角色：副主任；来源记载时点：2024-05-29；限制说明：原文未给实验室专名，不猜测。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P226" s="2" t="inlineStr"/>
+      <c r="Q226" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="R226" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S226" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>王子傲</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>工学博士</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr"/>
+      <c r="E227" s="2" t="inlineStr"/>
+      <c r="F227" s="2" t="inlineStr"/>
+      <c r="G227" s="2" t="inlineStr"/>
+      <c r="H227" s="2" t="inlineStr"/>
+      <c r="I227" s="2" t="inlineStr"/>
+      <c r="J227" s="2" t="inlineStr"/>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L227" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M227" s="2" t="inlineStr"/>
+      <c r="N227" s="2" t="inlineStr"/>
+      <c r="O227" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：工学博士；限制说明：官方主讲简介明确持有资格；哈工大为就业机构，不能当授位学校。。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P227" s="2" t="inlineStr"/>
+      <c r="Q227" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0330/c16314a341158/page.htm</t>
+        </is>
+      </c>
+      <c r="R227" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S227" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>王子傲</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>助理教授</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr"/>
+      <c r="F228" s="2" t="inlineStr"/>
+      <c r="G228" s="2" t="inlineStr"/>
+      <c r="H228" s="2" t="inlineStr"/>
+      <c r="I228" s="2" t="inlineStr"/>
+      <c r="J228" s="2" t="inlineStr"/>
+      <c r="K228" s="2" t="inlineStr"/>
+      <c r="L228" s="2" t="inlineStr"/>
+      <c r="M228" s="2" t="inlineStr"/>
+      <c r="N228" s="2" t="inlineStr"/>
+      <c r="O228" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；角色：助理教授；来源记载时点：2024-03-30。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P228" s="2" t="inlineStr"/>
+      <c r="Q228" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0330/c16314a341158/page.htm</t>
+        </is>
+      </c>
+      <c r="R228" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S228" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>双学士</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr"/>
+      <c r="F229" s="2" t="inlineStr"/>
+      <c r="G229" s="2" t="inlineStr"/>
+      <c r="H229" s="2" t="inlineStr"/>
+      <c r="I229" s="2" t="inlineStr"/>
+      <c r="J229" s="2" t="inlineStr"/>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L229" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M229" s="2" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="N229" s="2" t="inlineStr"/>
+      <c r="O229" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：双学士；机构：哈尔滨工业大学；来源学位数量：2；授位年份：2006；日期精度：年。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P229" s="2" t="inlineStr"/>
+      <c r="Q229" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R229" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S229" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr"/>
+      <c r="F230" s="2" t="inlineStr"/>
+      <c r="G230" s="2" t="inlineStr"/>
+      <c r="H230" s="2" t="inlineStr"/>
+      <c r="I230" s="2" t="inlineStr"/>
+      <c r="J230" s="2" t="inlineStr"/>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L230" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M230" s="2" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="N230" s="2" t="inlineStr"/>
+      <c r="O230" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：硕士；机构：哈尔滨工业大学；来源学位数量：1；授位年份：2008；日期精度：年。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P230" s="2" t="inlineStr"/>
+      <c r="Q230" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R230" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S230" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>普瓦提埃大学</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr"/>
+      <c r="F231" s="2" t="inlineStr"/>
+      <c r="G231" s="2" t="inlineStr"/>
+      <c r="H231" s="2" t="inlineStr"/>
+      <c r="I231" s="2" t="inlineStr"/>
+      <c r="J231" s="2" t="inlineStr"/>
+      <c r="K231" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L231" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M231" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="N231" s="2" t="inlineStr"/>
+      <c r="O231" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：博士；机构：普瓦提埃大学；来源学位数量：1；授位年份：2012；日期精度：年；国家原文：法国。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P231" s="2" t="inlineStr"/>
+      <c r="Q231" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R231" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S231" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院副院长、教授、博导</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr"/>
+      <c r="F232" s="2" t="inlineStr"/>
+      <c r="G232" s="2" t="inlineStr"/>
+      <c r="H232" s="2" t="inlineStr"/>
+      <c r="I232" s="2" t="inlineStr"/>
+      <c r="J232" s="2" t="inlineStr"/>
+      <c r="K232" s="2" t="inlineStr"/>
+      <c r="L232" s="2" t="inlineStr"/>
+      <c r="M232" s="2" t="inlineStr"/>
+      <c r="N232" s="2" t="inlineStr"/>
+      <c r="O232" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位：能源科学与工程学院；来源复合角色：能源科学与工程学院副院长、教授、博导；来源记载时点：2022-11-08；限制说明：教授/副院长为来源记载当时角色；博导是指导资格，非本人导师关系。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P232" s="2" t="inlineStr"/>
+      <c r="Q232" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R232" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S232" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>工作经历（职务未述）</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>CNRS-普瓦提埃大学</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr"/>
+      <c r="F233" s="2" t="inlineStr"/>
+      <c r="G233" s="2" t="inlineStr"/>
+      <c r="H233" s="2" t="inlineStr"/>
+      <c r="I233" s="2" t="inlineStr"/>
+      <c r="J233" s="2" t="inlineStr"/>
+      <c r="K233" s="2" t="inlineStr"/>
+      <c r="L233" s="2" t="inlineStr"/>
+      <c r="M233" s="2" t="inlineStr"/>
+      <c r="N233" s="2" t="inlineStr"/>
+      <c r="O233" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构原文：CNRS-普瓦提埃大学；原文次序：1；时间关系原文：2012年博士之后；依原文列举顺序，不编造分年起止。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P233" s="2" t="inlineStr"/>
+      <c r="Q233" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R233" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S233" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>工作经历（职务未述）</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>西班牙塞维利亚大学</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr"/>
+      <c r="F234" s="2" t="inlineStr"/>
+      <c r="G234" s="2" t="inlineStr"/>
+      <c r="H234" s="2" t="inlineStr"/>
+      <c r="I234" s="2" t="inlineStr"/>
+      <c r="J234" s="2" t="inlineStr"/>
+      <c r="K234" s="2" t="inlineStr"/>
+      <c r="L234" s="2" t="inlineStr"/>
+      <c r="M234" s="2" t="inlineStr"/>
+      <c r="N234" s="2" t="inlineStr"/>
+      <c r="O234" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构原文：西班牙塞维利亚大学；原文次序：2；时间关系原文：2012年博士之后；依原文列举顺序，不编造分年起止。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P234" s="2" t="inlineStr"/>
+      <c r="Q234" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R234" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S234" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>工作经历（职务未述）</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>CNRS-洛林大学</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr"/>
+      <c r="F235" s="2" t="inlineStr"/>
+      <c r="G235" s="2" t="inlineStr"/>
+      <c r="H235" s="2" t="inlineStr"/>
+      <c r="I235" s="2" t="inlineStr"/>
+      <c r="J235" s="2" t="inlineStr"/>
+      <c r="K235" s="2" t="inlineStr"/>
+      <c r="L235" s="2" t="inlineStr"/>
+      <c r="M235" s="2" t="inlineStr"/>
+      <c r="N235" s="2" t="inlineStr"/>
+      <c r="O235" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构原文：CNRS-洛林大学；原文次序：3；时间关系原文：2012年博士之后；依原文列举顺序，不编造分年起止。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P235" s="2" t="inlineStr"/>
+      <c r="Q235" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R235" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S235" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>工作经历（职务未述）</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr"/>
+      <c r="F236" s="2" t="inlineStr"/>
+      <c r="G236" s="2" t="inlineStr"/>
+      <c r="H236" s="2" t="inlineStr"/>
+      <c r="I236" s="2" t="inlineStr"/>
+      <c r="J236" s="2" t="inlineStr"/>
+      <c r="K236" s="2" t="inlineStr"/>
+      <c r="L236" s="2" t="inlineStr"/>
+      <c r="M236" s="2" t="inlineStr"/>
+      <c r="N236" s="2" t="inlineStr"/>
+      <c r="O236" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；事件年份：2017；限制说明：回国入职年，不等于教授/副院长职务开始年。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P236" s="2" t="inlineStr"/>
+      <c r="Q236" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="R236" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S236" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>西安交通大学</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr"/>
+      <c r="F237" s="2" t="inlineStr"/>
+      <c r="G237" s="2" t="inlineStr"/>
+      <c r="H237" s="2" t="inlineStr"/>
+      <c r="I237" s="2" t="inlineStr"/>
+      <c r="J237" s="2" t="inlineStr"/>
+      <c r="K237" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L237" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M237" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="N237" s="2" t="inlineStr"/>
+      <c r="O237" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：学士；机构：西安交通大学；来源学位数量：1；授位年份：2012；日期精度：年。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P237" s="2" t="inlineStr"/>
+      <c r="Q237" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/1029/c16314a357783/page.htm</t>
+        </is>
+      </c>
+      <c r="R237" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S237" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>西安交通大学</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr"/>
+      <c r="F238" s="2" t="inlineStr"/>
+      <c r="G238" s="2" t="inlineStr"/>
+      <c r="H238" s="2" t="inlineStr"/>
+      <c r="I238" s="2" t="inlineStr"/>
+      <c r="J238" s="2" t="inlineStr"/>
+      <c r="K238" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L238" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M238" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="N238" s="2" t="inlineStr"/>
+      <c r="O238" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：硕士；机构：西安交通大学；来源学位数量：1；授位年份：2015；日期精度：年。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P238" s="2" t="inlineStr"/>
+      <c r="Q238" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/1029/c16314a357783/page.htm</t>
+        </is>
+      </c>
+      <c r="R238" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S238" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>香港大学</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr"/>
+      <c r="F239" s="2" t="inlineStr"/>
+      <c r="G239" s="2" t="inlineStr"/>
+      <c r="H239" s="2" t="inlineStr"/>
+      <c r="I239" s="2" t="inlineStr"/>
+      <c r="J239" s="2" t="inlineStr"/>
+      <c r="K239" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L239" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M239" s="2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="N239" s="2" t="inlineStr"/>
+      <c r="O239" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：博士；机构：香港大学；来源学位数量：1；授位年份：2019；日期精度：年。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P239" s="2" t="inlineStr"/>
+      <c r="Q239" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/1029/c16314a357783/page.htm</t>
+        </is>
+      </c>
+      <c r="R239" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S239" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>能源学院教授、博导</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr"/>
+      <c r="F240" s="2" t="inlineStr"/>
+      <c r="G240" s="2" t="inlineStr"/>
+      <c r="H240" s="2" t="inlineStr"/>
+      <c r="I240" s="2" t="inlineStr"/>
+      <c r="J240" s="2" t="inlineStr"/>
+      <c r="K240" s="2" t="inlineStr"/>
+      <c r="L240" s="2" t="inlineStr"/>
+      <c r="M240" s="2" t="inlineStr"/>
+      <c r="N240" s="2" t="inlineStr"/>
+      <c r="O240" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位：能源学院；来源复合角色：能源学院教授、博导；来源记载时点：2024-10-29；限制说明：教授为来源记载当时角色；博导是指导资格，非本人导师关系。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P240" s="2" t="inlineStr"/>
+      <c r="Q240" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/1029/c16314a357783/page.htm</t>
+        </is>
+      </c>
+      <c r="R240" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S240" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S209"/>
+  <autoFilter ref="A1:S240"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -15412,6 +17453,37 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q207" r:id="rId207"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q208" r:id="rId208"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q209" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q210" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q211" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q212" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q213" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q214" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q215" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q216" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q217" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q218" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q219" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q220" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q221" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q222" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q223" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q224" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q225" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q226" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q227" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q228" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q229" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q230" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q231" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q232" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q233" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q234" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q235" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q236" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q237" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q238" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q239" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q240" r:id="rId240"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15423,7 +17495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -16146,8 +18218,62 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>蒲以康</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>来源博士论文目录导师</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：姓名：蒲以康；关系原文：导师；阶段：博士；限制说明：清华公开论文目录明确导师字段，未阅读论文原件。。同名、清华读博及等离子体方向的有界对应，不宣称独立唯一身份认证；未读取论文原件，仅绑定该博士学习记录，不确认授位；导师身份与当前任职未独立匹配。</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>来源目录关系，不提供人物身份或官方主页导航。</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>https://newetds.lib.tsinghua.edu.cn/qh/paper/summary?dbCode=ETDQH&amp;sysId=189075</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L13"/>
+  <autoFilter ref="A1:L14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
@@ -16161,6 +18287,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16172,17 +18299,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="50.4" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
     <col width="47.59999999999999" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="43.4" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
     <col width="65" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
@@ -18153,8 +20280,62 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>低温等离子体的发射光谱诊断与碰撞辐射模型研究</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>https://newetds.lib.tsinghua.edu.cn/qh/paper/summary?dbCode=ETDQH&amp;sysId=189075</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>博士论文（目录元数据）</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>https://newetds.lib.tsinghua.edu.cn/qh/paper/summary?dbCode=ETDQH&amp;sysId=189075</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>同名、清华读博及等离子体研究方向有界对应，非独立唯一身份认证。</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>公开目录元数据，未下载论文全文。</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：标题：低温等离子体的发射光谱诊断与碰撞辐射模型研究；英文标题：Investigation on the optical emission spectroscopy and the collisional-radiative model for the low-temperature plasmas；作者原序：朱悉铭；答辩日期：2009-12-24；机构：清华大学；页数：138；限制说明：目录书目元数据；答辩日期不是发表或授位日期，未下载全文。。答辩日期不是发表或授位日期；未下载全文，不认证学位获授。 同名、清华读博及等离子体方向有界对应，非独立唯一身份认证。</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L40"/>
+  <autoFilter ref="A1:L41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -18195,6 +20376,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18206,7 +20389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -22066,8 +24249,896 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>hit-changjuntao-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>https://news.hit.edu.cn/2025/0522/c1510a238003/page.htm</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_bodies_read_all_three</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>hit-changjuntao-official-2-20261030</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nwpu.edu.cn/info/1039/2890.htm</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_bodies_read_all_three</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>hit-changjuntao-official-3-20261030</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ncepu.edu.cn/xshd/f1015865691c45f6ac9b48dd423957e6.htm</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_bodies_read_all_three</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>hit-changjuntao-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>常军涛</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>hit-changjuntao-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhuximing-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>https://im.hit.edu.cn/en/2026/0318/c8918a388436/page.htm</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhuximing-official-2-20261030</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>https://newetds.lib.tsinghua.edu.cn/qh/paper/summary?dbCode=ETDQH&amp;sysId=189075</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhuximing-official-3-20261030</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>https://hitgs.hit.edu.cn/2017/0426/c17413a317511/page.htm</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhuximing-official-4-20261030</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>https://hitgs.hit.edu.cn/2018/0702/c17506a330002/page.htm</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhuximing-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>朱悉铭</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhuximing-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>hit-liuguodong-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0529/c16314a345683/page.htm</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>hit-liuguodong-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>刘国栋</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>hit-liuguodong-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>王子傲</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>hit-wangziao-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0330/c16314a341158/page.htm</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>王子傲</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>hit-wangziao-official-2-20261030</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>https://hituc.hit.edu.cn/2024/1106/c17860a358734/page.htm</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>王子傲</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>hit-wangziao-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>王子傲</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>hit-wangziao-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>hit-wujian-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2023/0919/c16297a327187/page.htm</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>hit-wujian-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>吴健</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>hit-wujian-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>hit-chaoyouchuang-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/1029/c16314a357783/page.htm</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>官方报道/通知/公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>hit-chaoyouchuang-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>晁攸闯</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>hit-chaoyouchuang-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G104"/>
+  <autoFilter ref="A1:G128"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -22172,6 +25243,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish eight accepted HIT official-source profiles with verified website and exports
</commit_message>
<xml_diff>
--- a/site/exports/hit-energy.xlsx
+++ b/site/exports/hit-energy.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$282</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,7 @@
     <col width="32.2" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="37.8" customWidth="1" min="7" max="7"/>
-    <col width="54.59999999999999" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
@@ -2477,8 +2477,432 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>教育为阶段/学位标签，未明确授位，来源未明确确认授位；不由学习结束年月推授位年月。；本人导师、博士教育未知。；2016历史页面至今仅保存当时语义，不认证2026当前任职。；原工作分段附带多个职务/称谓，不拆造各职务起止。；与魏显著合作招生不是本人师承。；来源记载职业信息：职业事实：参与项目数：10余项；论文数：30余篇；来源记载时点：2016-03-25。来源：https://power.hit.edu.cn/40/07/c5853a147463/page.psp；来源记载职业信息：职业事实：来源角色：中国动力工程学会水轮机专委会委员、全国海洋能转换设备标准化技术委员会委员、高等学校机电类学科教学委员会委员、黑龙江省机械工程学会液压与气动专业委员会副主任委员、《大电机技术》编委、Proceedings of the Institution of Mechanical Engineers, Part J, Journal of Engineering Tribology 审稿人；来源记载时点：2016-03-25。来源：https://power.hit.edu.cn/40/07/c5853a147463/page.psp；来源记载职业信息：职业事实：职业事实：负责4项国家科技支撑计划课题、负责1项国家科技重大专项子课题、负责哈尔滨大电机研究所新建实验台测控软件编写、负责多项校企合作横向课题；来源记载时点：2016-03-25。来源：https://power.hit.edu.cn/40/07/c5853a147463/page.psp；来源记载职业信息：职业事实：本科课程：工程流体力学、流体动力元件及控制系统；研究生课程：高等流体力学、流体机械及工程专题；精选教学荣誉：年份：2007；称谓：黑龙江省三育人先进工作者、年份：2008；称谓：力学课程教学团队国家级教学团队成员、年份：2009；称谓：工程流体力学国家精品课程负责人、年份：2009；称谓：热能动力类技术基础课程国家级教学团队成员、年份：2010；称谓：宝钢优秀教师奖；选取范围：职业/授课事实精选，并非逐条复制项目及全部教学奖项。；来源记载时点：2016-03-25。来源：https://power.hit.edu.cn/40/07/c5853a147463/page.psp；来源记载职业信息：职业事实：事实：与魏显著教授（兼职博导）合作招收博士生；限制说明：教学合作，不是本人导师关系。；来源记载时点：2016-03-25。来源：https://power.hit.edu.cn/40/07/c5853a147463/page.psp；来源记载职业信息：职业事实：单位原文：流体机械及工程研究所；角色：教授；职业称谓：教学带头人、省教学名师；来源记载时点：2016-03-25。所有统计、角色与今/至今以原来源时点为限，不认证2026当前在职；本人指导资格不作本人师承，不从博士后基金推本人在站。来源：https://power.hit.edu.cn/40/07/c5853a147463/page.psp；来源日期原标记：页面发布日期：2016-03-25；均为页面或文末来源时点，不是任职起止或本轮新近现职认证。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>官方历史院系教师资料：https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>三教育段仅学位/阶段标签，授位确认和授位日期未知。；工作与博士学习段原有重叠，原样保留，不改时间。；访问单位保持原名，不推国家或更名映射。；本人导师未知；硕士生导师是指导资格，不是本人师承。；今仅指2016历史来源时点，不认证2026在职。；来源记载职业信息：职业事实：项目总数：10；负责项目数：5；第一或第二作者论文数：11；SCI收录数：6；EI收录数：4；已授权发明专利数：7；限制说明：任职期间/来源当时统计；不扩大为当前总数，不从博士后基金推本人博士后任职。；来源记载时点：2016-03-25。来源：https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm；来源记载职业信息：职业事实：本科课程：气体放电及电推进技术（创新实验课）；研究生课程：等离子体物理、低温等离子体诊断技术；来源记载时点：2016-03-25。来源：https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm；来源日期原标记：页面发布日期：2016-03-25；均为页面或文末来源时点，不是任职起止或本轮新近现职认证。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>官方历史院系教师资料：https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>教育表为日期+阶段标签，不自补获授学位；武汉理工大学保源称，不追改历史校名。；至今仅2016来源口径，不认证2026任职。；只选前2作品，作者/卷页未列，不补造。科研项目未纳入本次精选范围。；来源记载职业信息：来源单位：动力机械振动与噪声控制技术研究所；来源角色：教授、博士生导师；原教育表：1980-09、1984-06、武汉理工大学、未述、船舶内燃机、学士、1985-09、1988-07、哈尔滨工业大学、能源学院、热力发动机、硕士、1992-03、1995-06、哈尔滨工业大学、能源学院、动力机械及工程、博士；原职业表：1988-07、1996-08、讲师、热力发动机、1996-08、1999-08、副教授、热力发动机、1999-08、至今、教授、热力发动机、1997-06、2000-06、硕士生导师、动力机械及工程、2000-06、至今、博士生导师、动力机械及工程；工作单位：哈尔滨工业大学；研究方向：转子动力学、动力机械振动与噪声控制、旋转机械故障诊断理论与技术、发动机结构强度与振动；学术服务：机构或期刊：中国振动工程学会；角色：常务理事、机构或期刊：中国振动工程学会转子动力学专业委员会；角色：主任委员；精选作品：原来源序号：1；标题：effects of shear stiffness in top foil structure on gas foil bearing performance based on thick plate theory；期刊：Proceedings of the Institution of Mechanical Engineers, Part J: Journal of Engineering Tribology；年份：2013、原来源序号：2；标题：A study of overall contact behavior of an elastic perfectly plastic hemisphere and a rigid plane；期刊：Proceedings of the Institution of Mechanical Engineers, Part J: Journal of Engineering Tribology；年份：2013；本科课程：发动机结构、发动机结构特点及核心技术、动力机械振动噪声控制技术前言及应用；研究生课程：转子动力学、故障诊断专家系统、高等转子动力学。所有统计、角色与今/至今以原来源时点为限，不认证2026当前在职；本人指导资格不作本人师承，不从博士后基金推本人在站。来源：https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm；来源日期原标记：页面发布日期：2016-03-25；均为页面或文末来源时点，不是任职起止或本轮新近现职认证。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>官方历史院系教师资料：https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>该能源领域何鹏与材料焊接领域同名教授不合并；未从同名材料页取职称。；简介列本人学位资格，未列授位年、导师或在职角色。；来源记载职业信息：来源资格院校：哈尔滨工业大学；来源资格学科：动力机械及工程；来源学位概述：学士、硕士、博士；非学位角色：博士后；非学位机构：英国诺丁汉大学罗罗传动技术中心；研究方向：转子动力学、接触、航发结构动力学、热弹耦合动力学；具体研究方向：复杂转子系统动力学、复杂结构热弹耦合动力学、粗糙表面接触动力学、重载滑动轴承热弹耦合分析；参与项目类型：国家自然科学基金、国家863燃机重大专项子课题、国防基础研究等课题；论文统计：合计：10；SCI收录数：3；EI收录数：5；单位：篇；范围限制：截至来源简介，SCI/EI是否重叠未知；具体书目原文：略。所有统计、角色与今/至今以原来源时点为限，不认证2026当前在职；本人指导资格不作本人师承，不从博士后基金推本人在站。来源：https://power.hit.edu.cn/81/60/c5853a164192/page.psp；来源日期原标记：页面发布日期：2016-07-28；均为页面或文末来源时点，不是任职起止或本轮新近现职认证。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。；仅能源领域何鹏；与材料焊接同名人物不合并，不移入其职称或教育。</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>官方历史院系教师资料：https://power.hit.edu.cn/81/60/c5853a164192/page.psp</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>本科/硕士经历、本人导师未知。；博士毕业年份与授位年份不混；毕业学校未知。；海外两校与访问/博士后类型未逐一对应。；从教20年为2024叙述相对时长，不倒推聘任起日。；来源记载职业信息：内容：2018年度入选国家级高层次人才计划；事件年份：2018。来源：https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm；来源记载职业信息：职业事实：从教时长原文：20年；本科竞赛指导时长原文：连续10余年；竞赛：全国大学生节能减排社会实践与科技竞赛；学生项目奖项：特等奖：3；一等奖：9；指导本科生提前毕业设计答辩人数：2；来源记载时点：2024-03-26；限制说明：教学指导及学生项目获奖，不当成本人学位、本人作品或研究生师承。。来源：https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm；来源事件年份：2003为博士毕业事件年，不是明确授位年份或页面日期；报道发表于2024-03-26，文末落款2024-03-24。历史来源不认证2026当前任职。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。；本条新增档案不改变唐天琪既有导师的阶段、人物身份或导航；不自动合并同名导师记录。</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>官方职业报道或报告人简介：https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>教育仅时间段+学位标签，授位确认/授位日期未知。；本人导师与专业未知，学院不是专业。；2009-12开始讲师与2008-12博士教育结束之间未提供经历，留空。；至今仅指2016来源时点，不推2026现职。；来源记载职业信息：精选项目：标题：霍尔推力器高电压下放电模式转变机理研究；资助方：国家自然科学基金；开始年份：2011；结束年份：2013；角色：负责人；选取范围：精选一个明确基础研究项目，未全采项目或技术摘要。。来源：https://power.hit.edu.cn/81/5a/c5853a164186/page.psp；来源日期原标记：页面发布日期：2016-07-28；均为页面或文末来源时点，不是任职起止或本轮新近现职认证。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>官方历史院系教师资料：https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>贺志宏</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>本科硕士经历与本人导师未见；博士后基金不能据此建立本人博士后经历；代表性文章仅写略，无具体作品可录；当前职位与任职终止未知，2016源职称不宣称当前认证；来源记载职业信息：研究方向：半透明材料电光热力耦合及调控机制、复杂形体内燃烧场辐射热环境数值仿真、多场耦合传热机制与并行计算、辐射传输、软硬电光材料光热传输及调控；主持项目：类型：国家自然科学基金；数量：1、类型：博士后基金；数量：1、类型：航天院所合作；原文数量：近5项；骨干参与项目：类型：自然科学面上项目；数量：3、类型：博士点基金；数量：1、类型：航天院所合作；原文数量：10余项；来源成果统计：论文数原文：20余篇；授权国家专利数：1；受理国家专利数：3；软件著作权数：2；合作领域：发动机燃烧及涡轮区辐射热环境仿真技术、软硬电光材料光热传输及调控技术、多场耦合传热机制与并行计算技术；代表性文章原文：略。所有统计、角色与今/至今以原来源时点为限，不认证2026当前在职；本人指导资格不作本人师承，不从博士后基金推本人在站。来源：https://power.hit.edu.cn/81/63/c5853a164195/page.psp；来源记载职业信息：角色：硕士生导师；来源记载时点：2016-07-28。所有统计、角色与今/至今以原来源时点为限，不认证2026当前在职；本人指导资格不作本人师承，不从博士后基金推本人在站。来源：https://power.hit.edu.cn/81/63/c5853a164195/page.psp；来源日期原标记：页面发布或更新日：2016-07-28；均为页面或文末来源时点，不是任职起止或本轮新近现职认证。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>官方历史院系教师资料：https://power.hit.edu.cn/81/63/c5853a164195/page.psp</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>郑智颖</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨校区</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>能源科学与工程学院</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 至 2026-10-30</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>授位院校/学科/年份及本人导师不明；师资博士后与博士资格分开；指导教师是本人指导职责，不是本人导师；仅2020-07-05更新来源记载师资博士后及指导职责，不认证当前在职；博士授位学校、专业、日期未知；来源日期原标记：页面发布或更新日：2020-07-05；均为页面或文末来源时点，不是任职起止或本轮新近现职认证。；既有名录2026-10-23仅姓名、单位及链接观察；本轮不重读、不修改原名录，不将旧主页链接升级已核个人主页。校区沿用既有能源学院harbin单位证据。；本批院校985、地域与洲不自动推补；明确国家仅按来源原文保留。</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>尚无本轮已核实个人主页；下列为官方历史学院教师简介、研究所介绍、职业报道、通知或公开书目资料，不是个人主页。</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>官方研究所团队资料：https://power.hit.edu.cn/_t881/16367/list.htm</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K38"/>
+  <autoFilter ref="A1:K46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -2521,7 +2945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S240"/>
+  <dimension ref="A1:S282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17241,8 +17665,2550 @@
         </is>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>1980-09</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>1984-07</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr"/>
+      <c r="H241" s="2" t="inlineStr"/>
+      <c r="I241" s="2" t="inlineStr"/>
+      <c r="J241" s="2" t="inlineStr"/>
+      <c r="K241" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L241" s="2" t="inlineStr"/>
+      <c r="M241" s="2" t="inlineStr"/>
+      <c r="N241" s="2" t="inlineStr"/>
+      <c r="O241" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1980-09；结束：1984-07；机构：哈尔滨工业大学；单位原文：能源学院动力工程系；称谓：学士；学习阶段：学士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P241" s="2" t="inlineStr"/>
+      <c r="Q241" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="R241" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S241" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>1984-08</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>1987-07</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr"/>
+      <c r="H242" s="2" t="inlineStr"/>
+      <c r="I242" s="2" t="inlineStr"/>
+      <c r="J242" s="2" t="inlineStr"/>
+      <c r="K242" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L242" s="2" t="inlineStr"/>
+      <c r="M242" s="2" t="inlineStr"/>
+      <c r="N242" s="2" t="inlineStr"/>
+      <c r="O242" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1984-08；结束：1987-07；机构：哈尔滨工业大学；单位原文：能源学院动力工程系；称谓：硕士；学习阶段：硕士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P242" s="2" t="inlineStr"/>
+      <c r="Q242" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="R242" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S242" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>助教</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>1987-08</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>1989-07</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr"/>
+      <c r="H243" s="2" t="inlineStr"/>
+      <c r="I243" s="2" t="inlineStr"/>
+      <c r="J243" s="2" t="inlineStr"/>
+      <c r="K243" s="2" t="inlineStr"/>
+      <c r="L243" s="2" t="inlineStr"/>
+      <c r="M243" s="2" t="inlineStr"/>
+      <c r="N243" s="2" t="inlineStr"/>
+      <c r="O243" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1987-08；结束：1989-07；单位：动力工程系；角色：助教；机构：哈尔滨工业大学；来源记载时点：2016-03-25；限制说明：时间段按原工作经历行保存，行内多角色不分别认证任期；至今只指来源时点。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P243" s="2" t="inlineStr"/>
+      <c r="Q243" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="R243" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S243" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>讲师</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>1989-08</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>1997-07</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr"/>
+      <c r="H244" s="2" t="inlineStr"/>
+      <c r="I244" s="2" t="inlineStr"/>
+      <c r="J244" s="2" t="inlineStr"/>
+      <c r="K244" s="2" t="inlineStr"/>
+      <c r="L244" s="2" t="inlineStr"/>
+      <c r="M244" s="2" t="inlineStr"/>
+      <c r="N244" s="2" t="inlineStr"/>
+      <c r="O244" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1989-08；结束：1997-07；单位：流体机械及工程；角色：讲师；机构：哈尔滨工业大学；来源记载时点：2016-03-25；限制说明：时间段按原工作经历行保存，行内多角色不分别认证任期；至今只指来源时点。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P244" s="2" t="inlineStr"/>
+      <c r="Q244" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="R244" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S244" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>副教授</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>1997-08</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>2006-08</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr"/>
+      <c r="H245" s="2" t="inlineStr"/>
+      <c r="I245" s="2" t="inlineStr"/>
+      <c r="J245" s="2" t="inlineStr"/>
+      <c r="K245" s="2" t="inlineStr"/>
+      <c r="L245" s="2" t="inlineStr"/>
+      <c r="M245" s="2" t="inlineStr"/>
+      <c r="N245" s="2" t="inlineStr"/>
+      <c r="O245" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1997-08；结束：2006-08；单位：流体机械及工程；角色：副教授；同段其他角色（不拆推任期）：流体机械教研室副主任、流体机械研究中心主任、能源学院飞行器推进及流体动力系副主任；机构：哈尔滨工业大学；来源记载时点：2016-03-25；限制说明：时间段按原工作经历行保存，行内多角色不分别认证任期；至今只指来源时点。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P245" s="2" t="inlineStr"/>
+      <c r="Q245" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="R245" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S245" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>2006-09</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr"/>
+      <c r="G246" s="2" t="inlineStr"/>
+      <c r="H246" s="2" t="inlineStr"/>
+      <c r="I246" s="2" t="inlineStr"/>
+      <c r="J246" s="2" t="inlineStr"/>
+      <c r="K246" s="2" t="inlineStr"/>
+      <c r="L246" s="2" t="inlineStr"/>
+      <c r="M246" s="2" t="inlineStr"/>
+      <c r="N246" s="2" t="inlineStr"/>
+      <c r="O246" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2006-09；结束原文：至今；单位：流体机械及工程；角色：教授；同段其他角色（不拆推任期）：副院长、教学带头人、省教学名师；机构：哈尔滨工业大学；来源记载时点：2016-03-25；限制说明：时间段按原工作经历行保存，行内多角色不分别认证任期；至今只指来源时点。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P246" s="2" t="inlineStr"/>
+      <c r="Q246" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="R246" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S246" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>1998-09</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>2002-07</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>热能与动力工程</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr"/>
+      <c r="I247" s="2" t="inlineStr"/>
+      <c r="J247" s="2" t="inlineStr"/>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L247" s="2" t="inlineStr"/>
+      <c r="M247" s="2" t="inlineStr"/>
+      <c r="N247" s="2" t="inlineStr"/>
+      <c r="O247" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1998-09；结束：2002-07；机构：哈尔滨工业大学；单位：能源学院；专业：热能与动力工程；学位阶段标签：学士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P247" s="2" t="inlineStr"/>
+      <c r="Q247" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R247" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S247" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>2002-09</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>2004-07</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>动力机械及工程</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr"/>
+      <c r="I248" s="2" t="inlineStr"/>
+      <c r="J248" s="2" t="inlineStr"/>
+      <c r="K248" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L248" s="2" t="inlineStr"/>
+      <c r="M248" s="2" t="inlineStr"/>
+      <c r="N248" s="2" t="inlineStr"/>
+      <c r="O248" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2002-09；结束：2004-07；机构：哈尔滨工业大学；单位：能源学院；专业：动力机械及工程；学位阶段标签：硕士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P248" s="2" t="inlineStr"/>
+      <c r="Q248" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R248" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S248" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>2004-09</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>2009-07</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>动力机械及工程</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr"/>
+      <c r="I249" s="2" t="inlineStr"/>
+      <c r="J249" s="2" t="inlineStr"/>
+      <c r="K249" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L249" s="2" t="inlineStr"/>
+      <c r="M249" s="2" t="inlineStr"/>
+      <c r="N249" s="2" t="inlineStr"/>
+      <c r="O249" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2004-09；结束：2009-07；机构：哈尔滨工业大学；单位：能源学院；专业：动力机械及工程；学位阶段标签：博士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P249" s="2" t="inlineStr"/>
+      <c r="Q249" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R249" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S249" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>visiting_scholar</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr"/>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>莫斯科国立无线电大学</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>2005-02</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>2006-01</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr"/>
+      <c r="H250" s="2" t="inlineStr"/>
+      <c r="I250" s="2" t="inlineStr"/>
+      <c r="J250" s="2" t="inlineStr"/>
+      <c r="K250" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L250" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M250" s="2" t="inlineStr"/>
+      <c r="N250" s="2" t="inlineStr"/>
+      <c r="O250" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2005-02；结束：2006-01；机构原文：莫斯科国立无线电大学；单位：等离子体光学系；角色：访问学者。非独立授位经历。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P250" s="2" t="inlineStr"/>
+      <c r="Q250" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R250" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S250" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>visiting_scholar</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr"/>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>中国科技大学</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>2010-09</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>2011-07</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr"/>
+      <c r="H251" s="2" t="inlineStr"/>
+      <c r="I251" s="2" t="inlineStr"/>
+      <c r="J251" s="2" t="inlineStr"/>
+      <c r="K251" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L251" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M251" s="2" t="inlineStr"/>
+      <c r="N251" s="2" t="inlineStr"/>
+      <c r="O251" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2010-09；结束：2011-07；机构原文：中国科技大学；单位：近代物理系；角色：访问学者。非独立授位经历。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P251" s="2" t="inlineStr"/>
+      <c r="Q251" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R251" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S251" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>助教</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>2004-09</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>2006-12</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr"/>
+      <c r="H252" s="2" t="inlineStr"/>
+      <c r="I252" s="2" t="inlineStr"/>
+      <c r="J252" s="2" t="inlineStr"/>
+      <c r="K252" s="2" t="inlineStr"/>
+      <c r="L252" s="2" t="inlineStr"/>
+      <c r="M252" s="2" t="inlineStr"/>
+      <c r="N252" s="2" t="inlineStr"/>
+      <c r="O252" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2004-09；结束：2006-12；角色：助教；机构：哈尔滨工业大学；单位原文：动力机械及工程学科；页头单位（非逐期任职单位认定）：先进动力控制研究所；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P252" s="2" t="inlineStr"/>
+      <c r="Q252" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R252" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S252" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>讲师</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>2006-12</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>2013-12</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr"/>
+      <c r="H253" s="2" t="inlineStr"/>
+      <c r="I253" s="2" t="inlineStr"/>
+      <c r="J253" s="2" t="inlineStr"/>
+      <c r="K253" s="2" t="inlineStr"/>
+      <c r="L253" s="2" t="inlineStr"/>
+      <c r="M253" s="2" t="inlineStr"/>
+      <c r="N253" s="2" t="inlineStr"/>
+      <c r="O253" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2006-12；结束：2013-12；角色：讲师；机构：哈尔滨工业大学；单位原文：动力机械及工程学科；页头单位（非逐期任职单位认定）：先进动力控制研究所；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P253" s="2" t="inlineStr"/>
+      <c r="Q253" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R253" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S253" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>硕士生导师</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>2011-06</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr"/>
+      <c r="G254" s="2" t="inlineStr"/>
+      <c r="H254" s="2" t="inlineStr"/>
+      <c r="I254" s="2" t="inlineStr"/>
+      <c r="J254" s="2" t="inlineStr"/>
+      <c r="K254" s="2" t="inlineStr"/>
+      <c r="L254" s="2" t="inlineStr"/>
+      <c r="M254" s="2" t="inlineStr"/>
+      <c r="N254" s="2" t="inlineStr"/>
+      <c r="O254" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2011-06；结束原文：今；角色：硕士生导师；机构：哈尔滨工业大学；单位原文：动力机械及工程学科；页头单位（非逐期任职单位认定）：先进动力控制研究所；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P254" s="2" t="inlineStr"/>
+      <c r="Q254" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R254" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S254" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>副教授</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>2014-01</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr"/>
+      <c r="G255" s="2" t="inlineStr"/>
+      <c r="H255" s="2" t="inlineStr"/>
+      <c r="I255" s="2" t="inlineStr"/>
+      <c r="J255" s="2" t="inlineStr"/>
+      <c r="K255" s="2" t="inlineStr"/>
+      <c r="L255" s="2" t="inlineStr"/>
+      <c r="M255" s="2" t="inlineStr"/>
+      <c r="N255" s="2" t="inlineStr"/>
+      <c r="O255" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2014-01；结束原文：今；角色：副教授；机构：哈尔滨工业大学；单位原文：动力机械及工程学科；页头单位（非逐期任职单位认定）：先进动力控制研究所；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P255" s="2" t="inlineStr"/>
+      <c r="Q255" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="R255" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S255" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>武汉理工大学</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>1980-09</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>1984-06</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>船舶内燃机</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr"/>
+      <c r="I256" s="2" t="inlineStr"/>
+      <c r="J256" s="2" t="inlineStr"/>
+      <c r="K256" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L256" s="2" t="inlineStr"/>
+      <c r="M256" s="2" t="inlineStr"/>
+      <c r="N256" s="2" t="inlineStr"/>
+      <c r="O256" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1980-09；结束：1984-06；机构：武汉理工大学；专业：船舶内燃机；来源层次：学士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P256" s="2" t="inlineStr"/>
+      <c r="Q256" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R256" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S256" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>1985-09</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>1988-07</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>热力发动机</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr"/>
+      <c r="I257" s="2" t="inlineStr"/>
+      <c r="J257" s="2" t="inlineStr"/>
+      <c r="K257" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L257" s="2" t="inlineStr"/>
+      <c r="M257" s="2" t="inlineStr"/>
+      <c r="N257" s="2" t="inlineStr"/>
+      <c r="O257" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1985-09；结束：1988-07；机构：哈尔滨工业大学；院系原文：能源学院；专业：热力发动机；来源层次：硕士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P257" s="2" t="inlineStr"/>
+      <c r="Q257" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R257" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S257" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>1992-03</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>1995-06</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>动力机械及工程</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr"/>
+      <c r="I258" s="2" t="inlineStr"/>
+      <c r="J258" s="2" t="inlineStr"/>
+      <c r="K258" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L258" s="2" t="inlineStr"/>
+      <c r="M258" s="2" t="inlineStr"/>
+      <c r="N258" s="2" t="inlineStr"/>
+      <c r="O258" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1992-03；结束：1995-06；机构：哈尔滨工业大学；院系原文：能源学院；专业：动力机械及工程；来源层次：博士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P258" s="2" t="inlineStr"/>
+      <c r="Q258" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R258" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S258" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>讲师</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>1988-07</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>1996-08</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr"/>
+      <c r="H259" s="2" t="inlineStr"/>
+      <c r="I259" s="2" t="inlineStr"/>
+      <c r="J259" s="2" t="inlineStr"/>
+      <c r="K259" s="2" t="inlineStr"/>
+      <c r="L259" s="2" t="inlineStr"/>
+      <c r="M259" s="2" t="inlineStr"/>
+      <c r="N259" s="2" t="inlineStr"/>
+      <c r="O259" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；起始：1988-07；结束：1996-08；结束原文：1996-08；角色：讲师；职业学科：热力发动机；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P259" s="2" t="inlineStr"/>
+      <c r="Q259" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R259" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S259" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>副教授</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>1996-08</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>1999-08</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr"/>
+      <c r="H260" s="2" t="inlineStr"/>
+      <c r="I260" s="2" t="inlineStr"/>
+      <c r="J260" s="2" t="inlineStr"/>
+      <c r="K260" s="2" t="inlineStr"/>
+      <c r="L260" s="2" t="inlineStr"/>
+      <c r="M260" s="2" t="inlineStr"/>
+      <c r="N260" s="2" t="inlineStr"/>
+      <c r="O260" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；起始：1996-08；结束：1999-08；结束原文：1999-08；角色：副教授；职业学科：热力发动机；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P260" s="2" t="inlineStr"/>
+      <c r="Q260" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R260" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S260" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>1999-08</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr"/>
+      <c r="G261" s="2" t="inlineStr"/>
+      <c r="H261" s="2" t="inlineStr"/>
+      <c r="I261" s="2" t="inlineStr"/>
+      <c r="J261" s="2" t="inlineStr"/>
+      <c r="K261" s="2" t="inlineStr"/>
+      <c r="L261" s="2" t="inlineStr"/>
+      <c r="M261" s="2" t="inlineStr"/>
+      <c r="N261" s="2" t="inlineStr"/>
+      <c r="O261" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；起始：1999-08；结束原文：至今；角色：教授；职业学科：热力发动机；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P261" s="2" t="inlineStr"/>
+      <c r="Q261" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R261" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S261" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>硕士生导师</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>1997-06</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>2000-06</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr"/>
+      <c r="H262" s="2" t="inlineStr"/>
+      <c r="I262" s="2" t="inlineStr"/>
+      <c r="J262" s="2" t="inlineStr"/>
+      <c r="K262" s="2" t="inlineStr"/>
+      <c r="L262" s="2" t="inlineStr"/>
+      <c r="M262" s="2" t="inlineStr"/>
+      <c r="N262" s="2" t="inlineStr"/>
+      <c r="O262" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；起始：1997-06；结束：2000-06；结束原文：2000-06；角色：硕士生导师；职业学科：动力机械及工程；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P262" s="2" t="inlineStr"/>
+      <c r="Q262" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R262" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S262" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>博士生导师</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>2000-06</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr"/>
+      <c r="G263" s="2" t="inlineStr"/>
+      <c r="H263" s="2" t="inlineStr"/>
+      <c r="I263" s="2" t="inlineStr"/>
+      <c r="J263" s="2" t="inlineStr"/>
+      <c r="K263" s="2" t="inlineStr"/>
+      <c r="L263" s="2" t="inlineStr"/>
+      <c r="M263" s="2" t="inlineStr"/>
+      <c r="N263" s="2" t="inlineStr"/>
+      <c r="O263" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；起始：2000-06；结束原文：至今；角色：博士生导师；职业学科：动力机械及工程；来源记载时点：2016-03-25。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P263" s="2" t="inlineStr"/>
+      <c r="Q263" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="R263" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S263" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr"/>
+      <c r="F264" s="2" t="inlineStr"/>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>动力机械及工程</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr"/>
+      <c r="I264" s="2" t="inlineStr"/>
+      <c r="J264" s="2" t="inlineStr"/>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L264" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M264" s="2" t="inlineStr"/>
+      <c r="N264" s="2" t="inlineStr"/>
+      <c r="O264" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：学士；机构：哈尔滨工业大学；专业：动力机械及工程。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P264" s="2" t="inlineStr"/>
+      <c r="Q264" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/60/c5853a164192/page.psp</t>
+        </is>
+      </c>
+      <c r="R264" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S264" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr"/>
+      <c r="F265" s="2" t="inlineStr"/>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>动力机械及工程</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr"/>
+      <c r="I265" s="2" t="inlineStr"/>
+      <c r="J265" s="2" t="inlineStr"/>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L265" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M265" s="2" t="inlineStr"/>
+      <c r="N265" s="2" t="inlineStr"/>
+      <c r="O265" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：硕士；机构：哈尔滨工业大学；专业：动力机械及工程。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P265" s="2" t="inlineStr"/>
+      <c r="Q265" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/60/c5853a164192/page.psp</t>
+        </is>
+      </c>
+      <c r="R265" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S265" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr"/>
+      <c r="F266" s="2" t="inlineStr"/>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>动力机械及工程</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr"/>
+      <c r="I266" s="2" t="inlineStr"/>
+      <c r="J266" s="2" t="inlineStr"/>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L266" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M266" s="2" t="inlineStr"/>
+      <c r="N266" s="2" t="inlineStr"/>
+      <c r="O266" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：博士；机构：哈尔滨工业大学；专业：动力机械及工程。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P266" s="2" t="inlineStr"/>
+      <c r="Q266" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/60/c5853a164192/page.psp</t>
+        </is>
+      </c>
+      <c r="R266" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S266" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>postdoctoral</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr"/>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>英国诺丁汉大学罗罗传动技术中心</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr"/>
+      <c r="F267" s="2" t="inlineStr"/>
+      <c r="G267" s="2" t="inlineStr"/>
+      <c r="H267" s="2" t="inlineStr"/>
+      <c r="I267" s="2" t="inlineStr"/>
+      <c r="J267" s="2" t="inlineStr"/>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L267" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M267" s="2" t="inlineStr"/>
+      <c r="N267" s="2" t="inlineStr"/>
+      <c r="O267" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构原文：英国诺丁汉大学罗罗传动技术中心。非独立授位经历。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P267" s="2" t="inlineStr"/>
+      <c r="Q267" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/60/c5853a164192/page.psp</t>
+        </is>
+      </c>
+      <c r="R267" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S267" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>graduation</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>博士毕业</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr"/>
+      <c r="E268" s="2" t="inlineStr"/>
+      <c r="F268" s="2" t="inlineStr"/>
+      <c r="G268" s="2" t="inlineStr"/>
+      <c r="H268" s="2" t="inlineStr"/>
+      <c r="I268" s="2" t="inlineStr"/>
+      <c r="J268" s="2" t="inlineStr"/>
+      <c r="K268" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L268" s="2" t="inlineStr"/>
+      <c r="M268" s="2" t="inlineStr"/>
+      <c r="N268" s="2" t="inlineStr"/>
+      <c r="O268" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：学习阶段：博士；来源层次：博士毕业；毕业年份（非授位年份推定）：2003；限制说明：博士毕业年明确，未明言授位/毕业学校；留校不自动补成HIT授位。。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P268" s="2" t="inlineStr"/>
+      <c r="Q268" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R268" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S268" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_research_combined</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr"/>
+      <c r="D269" s="2" t="inlineStr"/>
+      <c r="E269" s="2" t="inlineStr"/>
+      <c r="F269" s="2" t="inlineStr"/>
+      <c r="G269" s="2" t="inlineStr"/>
+      <c r="H269" s="2" t="inlineStr"/>
+      <c r="I269" s="2" t="inlineStr"/>
+      <c r="J269" s="2" t="inlineStr"/>
+      <c r="K269" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L269" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M269" s="2" t="inlineStr"/>
+      <c r="N269" s="2" t="inlineStr"/>
+      <c r="O269" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：并列机构原文（角色对应未述）：荷兰屯特大学、英国利兹大学；来源角色：访问学者、博士后研究；限制说明：两所大学与访问学者/博士后类别仅并列，逐校角色对应未知；合并保留，不拆造2个或4个明确角色事件。。非独立授位经历。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P269" s="2" t="inlineStr"/>
+      <c r="Q269" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R269" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S269" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr"/>
+      <c r="F270" s="2" t="inlineStr"/>
+      <c r="G270" s="2" t="inlineStr"/>
+      <c r="H270" s="2" t="inlineStr"/>
+      <c r="I270" s="2" t="inlineStr"/>
+      <c r="J270" s="2" t="inlineStr"/>
+      <c r="K270" s="2" t="inlineStr"/>
+      <c r="L270" s="2" t="inlineStr"/>
+      <c r="M270" s="2" t="inlineStr"/>
+      <c r="N270" s="2" t="inlineStr"/>
+      <c r="O270" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位原文：能源科学与工程学院；来源角色：教授；来源记载时点：2024-03-26。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P270" s="2" t="inlineStr"/>
+      <c r="Q270" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R270" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S270" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>留校工作</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr"/>
+      <c r="E271" s="2" t="inlineStr"/>
+      <c r="F271" s="2" t="inlineStr"/>
+      <c r="G271" s="2" t="inlineStr"/>
+      <c r="H271" s="2" t="inlineStr"/>
+      <c r="I271" s="2" t="inlineStr"/>
+      <c r="J271" s="2" t="inlineStr"/>
+      <c r="K271" s="2" t="inlineStr"/>
+      <c r="L271" s="2" t="inlineStr"/>
+      <c r="M271" s="2" t="inlineStr"/>
+      <c r="N271" s="2" t="inlineStr"/>
+      <c r="O271" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源角色：留校工作；事件年份：2003；限制说明：2003博士毕业留校工作原句，未独立标校名；不推教授聘任时间。。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P271" s="2" t="inlineStr"/>
+      <c r="Q271" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="R271" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S271" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>2003-09</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>2008-12</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr"/>
+      <c r="H272" s="2" t="inlineStr"/>
+      <c r="I272" s="2" t="inlineStr"/>
+      <c r="J272" s="2" t="inlineStr"/>
+      <c r="K272" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L272" s="2" t="inlineStr"/>
+      <c r="M272" s="2" t="inlineStr"/>
+      <c r="N272" s="2" t="inlineStr"/>
+      <c r="O272" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2003-09；结束：2008-12；机构：哈尔滨工业大学；单位：能源学院；称谓：博士；学习阶段：博士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P272" s="2" t="inlineStr"/>
+      <c r="Q272" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="R272" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S272" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>2001-09</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>2003-07</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr"/>
+      <c r="H273" s="2" t="inlineStr"/>
+      <c r="I273" s="2" t="inlineStr"/>
+      <c r="J273" s="2" t="inlineStr"/>
+      <c r="K273" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L273" s="2" t="inlineStr"/>
+      <c r="M273" s="2" t="inlineStr"/>
+      <c r="N273" s="2" t="inlineStr"/>
+      <c r="O273" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2001-09；结束：2003-07；机构：哈尔滨工业大学；单位：能源学院；称谓：硕士；学习阶段：硕士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P273" s="2" t="inlineStr"/>
+      <c r="Q273" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="R273" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S273" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学（威海）</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>1997-09</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>2001-07</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr"/>
+      <c r="H274" s="2" t="inlineStr"/>
+      <c r="I274" s="2" t="inlineStr"/>
+      <c r="J274" s="2" t="inlineStr"/>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L274" s="2" t="inlineStr"/>
+      <c r="M274" s="2" t="inlineStr"/>
+      <c r="N274" s="2" t="inlineStr"/>
+      <c r="O274" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：1997-09；结束：2001-07；机构：哈尔滨工业大学（威海）；单位：汽车学院；称谓：学士；学习阶段：学士。来源学习阶段不确认授位。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P274" s="2" t="inlineStr"/>
+      <c r="Q274" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="R274" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S274" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>副教授</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>2015-01</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr"/>
+      <c r="G275" s="2" t="inlineStr"/>
+      <c r="H275" s="2" t="inlineStr"/>
+      <c r="I275" s="2" t="inlineStr"/>
+      <c r="J275" s="2" t="inlineStr"/>
+      <c r="K275" s="2" t="inlineStr"/>
+      <c r="L275" s="2" t="inlineStr"/>
+      <c r="M275" s="2" t="inlineStr"/>
+      <c r="N275" s="2" t="inlineStr"/>
+      <c r="O275" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2015-01；结束原文：至今；机构：哈尔滨工业大学；单位：能源学院；角色：副教授；来源记载时点：2016-07-28。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P275" s="2" t="inlineStr"/>
+      <c r="Q275" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="R275" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S275" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>讲师</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>2009-12</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>2014-12</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr"/>
+      <c r="H276" s="2" t="inlineStr"/>
+      <c r="I276" s="2" t="inlineStr"/>
+      <c r="J276" s="2" t="inlineStr"/>
+      <c r="K276" s="2" t="inlineStr"/>
+      <c r="L276" s="2" t="inlineStr"/>
+      <c r="M276" s="2" t="inlineStr"/>
+      <c r="N276" s="2" t="inlineStr"/>
+      <c r="O276" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：起始：2009-12；结束：2014-12；机构：哈尔滨工业大学；单位：能源学院；角色：讲师；来源记载时点：2016-07-28。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P276" s="2" t="inlineStr"/>
+      <c r="Q276" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="R276" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S276" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>贺志宏</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr"/>
+      <c r="F277" s="2" t="inlineStr"/>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>工程热物理</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="inlineStr"/>
+      <c r="I277" s="2" t="inlineStr"/>
+      <c r="J277" s="2" t="inlineStr"/>
+      <c r="K277" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L277" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M277" s="2" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="N277" s="2" t="inlineStr"/>
+      <c r="O277" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：博士；机构：哈尔滨工业大学；专业：工程热物理；授位年份：2001；毕业年份（非授位年份推定）：2001。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P277" s="2" t="inlineStr"/>
+      <c r="Q277" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/63/c5853a164195/page.psp</t>
+        </is>
+      </c>
+      <c r="R277" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S277" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>贺志宏</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>副教授</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr"/>
+      <c r="F278" s="2" t="inlineStr"/>
+      <c r="G278" s="2" t="inlineStr"/>
+      <c r="H278" s="2" t="inlineStr"/>
+      <c r="I278" s="2" t="inlineStr"/>
+      <c r="J278" s="2" t="inlineStr"/>
+      <c r="K278" s="2" t="inlineStr"/>
+      <c r="L278" s="2" t="inlineStr"/>
+      <c r="M278" s="2" t="inlineStr"/>
+      <c r="N278" s="2" t="inlineStr"/>
+      <c r="O278" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位原文：能源学院；标题：副教授；来源记载时点：2016-07-28。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P278" s="2" t="inlineStr"/>
+      <c r="Q278" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/63/c5853a164195/page.psp</t>
+        </is>
+      </c>
+      <c r="R278" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S278" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>贺志宏</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>留校任教</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr"/>
+      <c r="F279" s="2" t="inlineStr"/>
+      <c r="G279" s="2" t="inlineStr"/>
+      <c r="H279" s="2" t="inlineStr"/>
+      <c r="I279" s="2" t="inlineStr"/>
+      <c r="J279" s="2" t="inlineStr"/>
+      <c r="K279" s="2" t="inlineStr"/>
+      <c r="L279" s="2" t="inlineStr"/>
+      <c r="M279" s="2" t="inlineStr"/>
+      <c r="N279" s="2" t="inlineStr"/>
+      <c r="O279" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；角色：留校任教；限制说明：2001年留校任教事件；不推副教授、硕士生导师或其他职务聘期。；事件年份：2001。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P279" s="2" t="inlineStr"/>
+      <c r="Q279" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/63/c5853a164195/page.psp</t>
+        </is>
+      </c>
+      <c r="R279" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S279" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>郑智颖</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr"/>
+      <c r="E280" s="2" t="inlineStr"/>
+      <c r="F280" s="2" t="inlineStr"/>
+      <c r="G280" s="2" t="inlineStr"/>
+      <c r="H280" s="2" t="inlineStr"/>
+      <c r="I280" s="2" t="inlineStr"/>
+      <c r="J280" s="2" t="inlineStr"/>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L280" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M280" s="2" t="inlineStr"/>
+      <c r="N280" s="2" t="inlineStr"/>
+      <c r="O280" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：来源学位称谓：博士。来源明确记载获授或持有资格；非证书核验。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。</t>
+        </is>
+      </c>
+      <c r="P280" s="2" t="inlineStr"/>
+      <c r="Q280" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/_t881/16367/list.htm</t>
+        </is>
+      </c>
+      <c r="R280" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S280" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>郑智颖</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>postdoctoral</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr"/>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr"/>
+      <c r="F281" s="2" t="inlineStr"/>
+      <c r="G281" s="2" t="inlineStr"/>
+      <c r="H281" s="2" t="inlineStr"/>
+      <c r="I281" s="2" t="inlineStr"/>
+      <c r="J281" s="2" t="inlineStr"/>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L281" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M281" s="2" t="inlineStr"/>
+      <c r="N281" s="2" t="inlineStr"/>
+      <c r="O281" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学。非独立授位经历。学习起止不由授位、答辩或事件时间推定；不据校名推地域分类。 与同源职业栏师资博士后是同一角色的非学位表达，不是第二次独立在站；博士资格授位院校不因HIT任职而补成HIT。</t>
+        </is>
+      </c>
+      <c r="P281" s="2" t="inlineStr"/>
+      <c r="Q281" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/_t881/16367/list.htm</t>
+        </is>
+      </c>
+      <c r="R281" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S281" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>郑智颖</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>指导教师/师资博士后</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr"/>
+      <c r="F282" s="2" t="inlineStr"/>
+      <c r="G282" s="2" t="inlineStr"/>
+      <c r="H282" s="2" t="inlineStr"/>
+      <c r="I282" s="2" t="inlineStr"/>
+      <c r="J282" s="2" t="inlineStr"/>
+      <c r="K282" s="2" t="inlineStr"/>
+      <c r="L282" s="2" t="inlineStr"/>
+      <c r="M282" s="2" t="inlineStr"/>
+      <c r="N282" s="2" t="inlineStr"/>
+      <c r="O282" s="2" t="inlineStr">
+        <is>
+          <t>来源记载：机构：哈尔滨工业大学；单位原文：流体机械及工程研究所；课题组原文：复杂流动与传热课题组；来源角色：指导教师/师资博士后；来源记载时点：2020-07-05。任职起止未明确者保留未知；历史来源角色不认证2026当前在职；博导等仅本人指导资格，不转成本人导师。</t>
+        </is>
+      </c>
+      <c r="P282" s="2" t="inlineStr"/>
+      <c r="Q282" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/_t881/16367/list.htm</t>
+        </is>
+      </c>
+      <c r="R282" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="S282" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S240"/>
+  <autoFilter ref="A1:S282"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -17484,6 +20450,48 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q238" r:id="rId238"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q239" r:id="rId239"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q240" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q241" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q242" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q243" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q244" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q245" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q246" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q247" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q248" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q249" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q250" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q251" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q252" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q253" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q254" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q255" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q256" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q257" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q258" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q259" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q260" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q261" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q262" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q263" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q264" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q265" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q266" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q267" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q268" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q269" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q270" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q271" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q272" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q273" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q274" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q275" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q276" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q277" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q278" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q279" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q280" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q281" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q282" r:id="rId282"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18299,7 +21307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -20334,8 +23342,440 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Application of Entropy Production Theory in Hydro-turbine Hydraulic Analysis.</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：1；作者原顺序：Ru-Zhi Gong、Hong-Jie Wang、Li-Xia Chen、De-You Li、Hao-Chun Zhang、Xian-Zhu Wei；标题：Application of Entropy Production Theory in Hydro-turbine Hydraulic Analysis.；期刊：SCIENCE CHINA Technological Sciences；年份：2013；卷：56；期：7；页数：1636-1643；来源角色：通讯作者。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Influence of clearance parameters on the rotor dynamic character of hydraulic turbine shaft system.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：2；作者原顺序：Ru-Zhi Gong、Hong-Jie Wang、Jun-Long Zhao、De-You Li、Xian-Zhu Wei；标题：Influence of clearance parameters on the rotor dynamic character of hydraulic turbine shaft system.；期刊：Proceedings of the Institution of Mechanical Engineers, Part C, Journal of Mechanical Engineering and Science；年份：2014；卷：228；期：2；页数：262-270；来源角色：通讯作者。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Effects of ionization distribution on plasma beam focusingcharacteristics in Hall thrusters.</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：1；作者原顺序：Zhongxi Ning、Hui Liu、Daren Yu、Zhongxiang Zhou；题名原文：Effects of ionization distribution on plasma beam focusingcharacteristics in Hall thrusters.；期刊：APPLIED PHYSICS LETTERS；卷：99；年份：2011；文章号：221502；限制说明：focusingcharacteristics原抽取连字保留，未静默修正。。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>On the frequency characteristic of inductor in the filter of Hall thrusters.</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：2；作者原顺序：Wei Liqiu、Ning Zhongxi、E. Peng、Yu Daren；标题：On the frequency characteristic of inductor in the filter of Hall thrusters.；期刊：J. Vac. Sci. Technol.；年份：2010；系列：A；卷：28；期：5；页码原文：L9。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>effects of shear stiffness in top foil structure on gas foil bearing performance based on thick plate theory</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：1；标题：effects of shear stiffness in top foil structure on gas foil bearing performance based on thick plate theory；期刊：Proceedings of the Institution of Mechanical Engineers, Part J: Journal of Engineering Tribology；年份：2013。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>A study of overall contact behavior of an elastic perfectly plastic hemisphere and a rigid plane</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：2；标题：A study of overall contact behavior of an elastic perfectly plastic hemisphere and a rigid plane；期刊：Proceedings of the Institution of Mechanical Engineers, Part J: Journal of Engineering Tribology；年份：2013。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Relationship between magnetic field strength and discharge voltage of ATON-type Hall thrusters.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：1；作者原顺序：Ding, Y. J.、Wei, L. Q.、Jia, D. C.；标题：Relationship between magnetic field strength and discharge voltage of ATON-type Hall thrusters.；期刊：PHYSICA SCRIPTA；年份：2014；卷：89；期：8；文章号：085602。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Scaling Design and Experimental Study on Hall Thrusters with Curved Magnetic Field</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：2；作者原顺序：Ding, Y. J.、Yu, D. R.、Jia, D. C.、Yan, G. J.、Li, H.；标题：Scaling Design and Experimental Study on Hall Thrusters with Curved Magnetic Field；期刊：Contributions to Plasma Physics；年份：2011；卷：51；期：1；页数：68-82。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>空间电推进原理</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>著作；book</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>来源书目：原来源序号：8；类型：book；作者原顺序：于达仁、刘辉、丁永杰、宁中喜、魏立秋；标题：空间电推进原理；出版社：哈尔滨工业大学出版社；年份：2014；限制说明：原书条为[8]，条内另有“14、”前缀；保留原异常，source_order仍为8，不纠正为第14项。。原作者顺序、拼写及书目序号保留；仅官方页面书目，未核出版商或全文，不推作者身份、导师关系或排名。</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L41"/>
+  <autoFilter ref="A1:L50"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -20378,6 +23818,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20389,7 +23838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G128"/>
+  <dimension ref="A1:G152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -25137,8 +28586,896 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>hit-wanghongjie-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/40/07/c5853a147463/page.psp</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>hit-wanghongjie-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>王洪杰</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>hit-wanghongjie-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>hit-ningzhongxi-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147490/page.htm</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>hit-ningzhongxi-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>宁中喜</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>hit-ningzhongxi-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>hit-liuzhansheng-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/2016/0325/c5853a147464/page.htm</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>hit-liuzhansheng-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>刘占生</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>hit-liuzhansheng-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>hit-hepeng-energy-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/60/c5853a164192/page.psp</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>hit-hepeng-energy-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>何鹏</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>hit-hepeng-energy-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>hit-heyurong-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>https://future.hit.edu.cn/2024/0326/c16314a340786/page.htm</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>hit-heyurong-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>何玉荣</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>hit-heyurong-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>hit-dingyongjie-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/5a/c5853a164186/page.psp</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_official_article_and_public_metadata_bodies_read</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>hit-dingyongjie-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>丁永杰</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>hit-dingyongjie-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>贺志宏</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>hit-hezhihong-energy-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/81/63/c5853a164195/page.psp</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_exact_official_body_read</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>贺志宏</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>hit-hezhihong-energy-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>贺志宏</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>hit-hezhihong-energy-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>郑智颖</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhengzhiying-energy-official-1-20261030</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/_t881/16367/list.htm</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>官方历史学院教师简介、研究所介绍、报道、通知或公开目录有界复读，非个人主页或当前人事认证。；independent_normal_web_exact_official_body_read</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>郑智颖</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhengzhiying-energy-roster-20261023</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/5735/list.htm</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>郑智颖</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>hit-zhengzhiying-energy-campus-20261023</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>https://power.hit.edu.cn/</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>沿用既有单位和名录观察，非本轮新读或个人主页认证。</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>哈尔滨工业大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G128"/>
+  <autoFilter ref="A1:G152"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -25267,6 +29604,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId151"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>